<commit_message>
test(auth): implement TC_LOGIN_03 for non-existent account verification
</commit_message>
<xml_diff>
--- a/test-data/LoginTestCases.xlsx
+++ b/test-data/LoginTestCases.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -577,6 +577,43 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Đăng nhập thất bại do tài khoản không tồn tại trên hệ thống</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>unknown_account_xyz</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>AnyPassword@123</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Ở lại trang đăng nhập, hiển thị thông báo tài khoản không tồn tại</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống từ chối xác thực tài khoản không tồn tại</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test(auth): implement TC_LOGIN_02 for invalid password authentication failure
</commit_message>
<xml_diff>
--- a/test-data/LoginTestCases.xlsx
+++ b/test-data/LoginTestCases.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -540,6 +540,43 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_02</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Đăng nhập thất bại do nhập sai mật khẩu</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>student_test</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>WrongPassword!99</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Ở lại trang đăng nhập, hiển thị thông báo lỗi sai thông tin</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống từ chối truy cập và ở lại trang đăng nhập do sai mật khẩu</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test(auth): implement TC_LOGIN_01 for valid credentials happy path flow
</commit_message>
<xml_diff>
--- a/test-data/LoginTestCases.xlsx
+++ b/test-data/LoginTestCases.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,6 +29,12 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00008000"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -46,7 +52,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -54,14 +60,34 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D3D3D3"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D3D3D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D3D3D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D3D3D3"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -428,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -477,6 +503,43 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Đăng nhập thành công với thông tin tài khoản hợp lệ</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>student_test</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Utc@2026Password</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Rời khỏi trang đăng nhập, chuyển hướng đến trang chủ / Dashboard</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Chuyển hướng thành công tới hệ thống, URL: https://vanphongdientu.utc.edu.vn/Login</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test(validation): implement TC_LOGIN_04 for empty credentials validation
</commit_message>
<xml_diff>
--- a/test-data/LoginTestCases.xlsx
+++ b/test-data/LoginTestCases.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -614,6 +614,35 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_04</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Bỏ trống cả Tên đăng nhập và Mật khẩu (Validation)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Không cho phép gửi form, hiển thị cảnh báo yêu cầu nhập thông tin</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Không cho phép gửi form rỗng, hiển thị cảnh báo validation</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test(validation): implement TC_LOGIN_06 for missing username validation
</commit_message>
<xml_diff>
--- a/test-data/LoginTestCases.xlsx
+++ b/test-data/LoginTestCases.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -676,6 +676,39 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_06</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Bỏ trống Tên đăng nhập nhưng có nhập Mật khẩu</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Utc@2026Password</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Không cho phép gửi form, hiển thị cảnh báo yêu cầu nhập tên đăng nhập</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Chặn gửi form rỗng tên đăng nhập, hiển thị cảnh báo hợp lệ</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test(ui): implement TC_LOGIN_07 for remember me checkbox interaction
</commit_message>
<xml_diff>
--- a/test-data/LoginTestCases.xlsx
+++ b/test-data/LoginTestCases.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -709,6 +709,43 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_07</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Đăng nhập kèm tích chọn tùy chọn Ghi nhớ đăng nhập</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>student_test</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Utc@2026Password</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Tích chọn checkbox ghi nhớ và gửi yêu cầu đăng nhập hợp lệ</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Tích chọn ghi nhớ thành công và gửi dữ liệu đăng nhập hợp lệ</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test(validation): implement TC_LOGIN_05 for missing password validation
</commit_message>
<xml_diff>
--- a/test-data/LoginTestCases.xlsx
+++ b/test-data/LoginTestCases.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -643,6 +643,39 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_05</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Nhập Tên đăng nhập nhưng bỏ trống Mật khẩu (Slide Buổi 8)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>student_test</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Không cho phép gửi form, hiển thị cảnh báo yêu cầu nhập mật khẩu</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Chặn gửi form rỗng mật khẩu, hiển thị cảnh báo hợp lệ</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test(security): implement TC_LOGIN_08 for SQL injection payload sanitization
</commit_message>
<xml_diff>
--- a/test-data/LoginTestCases.xlsx
+++ b/test-data/LoginTestCases.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -746,6 +746,43 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_08</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Kiểm tra bảo mật phòng chống tấn công SQL Injection</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>' OR '1'='1</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>' OR '1'='1</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống ngăn chặn payload SQL và từ chối xác thực an toàn</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống ngăn chặn chuỗi payload SQL Injection an toàn</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(report): integrate Allure Report and automatic failure screenshot attachments
</commit_message>
<xml_diff>
--- a/test-data/LoginTestCases.xlsx
+++ b/test-data/LoginTestCases.xlsx
@@ -9,15 +9,18 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LoginTestCases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="0" uniqueCount="0"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +39,54 @@
       <b val="1"/>
       <color rgb="00008000"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
     </font>
   </fonts>
   <fills count="3">
@@ -78,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -89,6 +140,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -457,13 +516,13 @@
   <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col min="1" max="1" customWidth="true" width="16.0"/>
+    <col min="2" max="2" customWidth="true" width="46.0"/>
+    <col min="3" max="3" customWidth="true" width="24.0"/>
+    <col min="4" max="4" customWidth="true" width="24.0"/>
+    <col min="5" max="5" customWidth="true" width="52.0"/>
+    <col min="6" max="6" customWidth="true" width="38.0"/>
+    <col min="7" max="7" customWidth="true" width="14.0"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -530,11 +589,13 @@
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
+        <v>Chuyển hướng thành công tới hệ thống, URL: https://vanphongdientu.utc.edu.vn/Login (Thông báo UI: Tài khoản hoặc mật khẩu không đúng.)</v>
         <is>
           <t>Chuyển hướng thành công tới hệ thống, URL: https://vanphongdientu.utc.edu.vn/Login</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
+        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -567,11 +628,13 @@
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
+        <v>Hệ thống từ chối truy cập và ở lại trang đăng nhập do sai mật khẩu (Thông báo UI: Tài khoản hoặc mật khẩu không đúng.)</v>
         <is>
           <t>Hệ thống từ chối truy cập và ở lại trang đăng nhập do sai mật khẩu</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
+        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -604,11 +667,13 @@
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
+        <v>Hệ thống từ chối xác thực tài khoản không tồn tại (Thông báo UI: Tài khoản hoặc mật khẩu không đúng.)</v>
         <is>
           <t>Hệ thống từ chối xác thực tài khoản không tồn tại</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
+        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -633,11 +698,13 @@
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
+        <v>Không cho phép gửi form rỗng, hiển thị cảnh báo validation (Thông báo UI: Bạn chưa nhập tên đăng nhập)</v>
         <is>
           <t>Không cho phép gửi form rỗng, hiển thị cảnh báo validation</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
+        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -666,11 +733,13 @@
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
+        <v>Chặn gửi form rỗng mật khẩu, hiển thị cảnh báo hợp lệ (Thông báo UI: Bạn chưa nhập mật khẩu)</v>
         <is>
           <t>Chặn gửi form rỗng mật khẩu, hiển thị cảnh báo hợp lệ</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="8" t="inlineStr">
+        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -699,11 +768,13 @@
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
+        <v>Chặn gửi form rỗng tên đăng nhập, hiển thị cảnh báo hợp lệ (Thông báo UI: Bạn chưa nhập tên đăng nhập)</v>
         <is>
           <t>Chặn gửi form rỗng tên đăng nhập, hiển thị cảnh báo hợp lệ</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="9" t="inlineStr">
+        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -736,11 +807,13 @@
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
+        <v>Tích chọn ghi nhớ thành công và gửi dữ liệu đăng nhập hợp lệ (Thông báo UI: Tài khoản hoặc mật khẩu không đúng.)</v>
         <is>
           <t>Tích chọn ghi nhớ thành công và gửi dữ liệu đăng nhập hợp lệ</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="10" t="inlineStr">
+        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -773,11 +846,13 @@
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
+        <v>Hệ thống ngăn chặn chuỗi payload SQL Injection an toàn (Thông báo UI: Tài khoản hoặc mật khẩu không đúng.)</v>
         <is>
           <t>Hệ thống ngăn chặn chuỗi payload SQL Injection an toàn</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G9" s="11" t="inlineStr">
+        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>

</xml_diff>

<commit_message>
test(security): implement TC_LOGIN_09 for XSS script payload sanitization
</commit_message>
<xml_diff>
--- a/test-data/LoginTestCases.xlsx
+++ b/test-data/LoginTestCases.xlsx
@@ -9,12 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LoginTestCases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="0" uniqueCount="0"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -42,51 +39,51 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
+      <b val="1"/>
       <color indexed="17"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color indexed="17"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color indexed="17"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color indexed="17"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color indexed="17"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color indexed="17"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color indexed="17"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color indexed="17"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -129,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -140,14 +137,20 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -513,16 +516,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="16.0"/>
-    <col min="2" max="2" customWidth="true" width="46.0"/>
-    <col min="3" max="3" customWidth="true" width="24.0"/>
-    <col min="4" max="4" customWidth="true" width="24.0"/>
-    <col min="5" max="5" customWidth="true" width="52.0"/>
-    <col min="6" max="6" customWidth="true" width="38.0"/>
-    <col min="7" max="7" customWidth="true" width="14.0"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -589,13 +592,11 @@
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
-        <v>Chuyển hướng thành công tới hệ thống, URL: https://vanphongdientu.utc.edu.vn/Login (Thông báo UI: Tài khoản hoặc mật khẩu không đúng.)</v>
         <is>
           <t>Chuyển hướng thành công tới hệ thống, URL: https://vanphongdientu.utc.edu.vn/Login</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
-        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -628,13 +629,11 @@
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
-        <v>Hệ thống từ chối truy cập và ở lại trang đăng nhập do sai mật khẩu (Thông báo UI: Tài khoản hoặc mật khẩu không đúng.)</v>
         <is>
           <t>Hệ thống từ chối truy cập và ở lại trang đăng nhập do sai mật khẩu</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
-        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -667,13 +666,11 @@
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
-        <v>Hệ thống từ chối xác thực tài khoản không tồn tại (Thông báo UI: Tài khoản hoặc mật khẩu không đúng.)</v>
         <is>
           <t>Hệ thống từ chối xác thực tài khoản không tồn tại</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
-        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -698,13 +695,11 @@
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
-        <v>Không cho phép gửi form rỗng, hiển thị cảnh báo validation (Thông báo UI: Bạn chưa nhập tên đăng nhập)</v>
         <is>
           <t>Không cho phép gửi form rỗng, hiển thị cảnh báo validation</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
-        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -733,13 +728,11 @@
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
-        <v>Chặn gửi form rỗng mật khẩu, hiển thị cảnh báo hợp lệ (Thông báo UI: Bạn chưa nhập mật khẩu)</v>
         <is>
           <t>Chặn gửi form rỗng mật khẩu, hiển thị cảnh báo hợp lệ</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
-        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -768,13 +761,11 @@
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
-        <v>Chặn gửi form rỗng tên đăng nhập, hiển thị cảnh báo hợp lệ (Thông báo UI: Bạn chưa nhập tên đăng nhập)</v>
         <is>
           <t>Chặn gửi form rỗng tên đăng nhập, hiển thị cảnh báo hợp lệ</t>
         </is>
       </c>
       <c r="G7" s="9" t="inlineStr">
-        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -807,13 +798,11 @@
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
-        <v>Tích chọn ghi nhớ thành công và gửi dữ liệu đăng nhập hợp lệ (Thông báo UI: Tài khoản hoặc mật khẩu không đúng.)</v>
         <is>
           <t>Tích chọn ghi nhớ thành công và gửi dữ liệu đăng nhập hợp lệ</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
-        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -846,13 +835,48 @@
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
-        <v>Hệ thống ngăn chặn chuỗi payload SQL Injection an toàn (Thông báo UI: Tài khoản hoặc mật khẩu không đúng.)</v>
         <is>
           <t>Hệ thống ngăn chặn chuỗi payload SQL Injection an toàn</t>
         </is>
       </c>
       <c r="G9" s="11" t="inlineStr">
-        <v>PASS</v>
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_09</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Kiểm tra bảo mật chống tấn công Cross-Site Scripting (XSS)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>&lt;script&gt;alert('XSS')&lt;/script&gt;</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>TestPassword@123</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống ngăn chặn mã script độc hại, giữ an toàn tại trang đăng nhập</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống xử lý an toàn chuỗi XSS payload và từ chối xác thực</t>
+        </is>
+      </c>
+      <c r="G10" s="13" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>

</xml_diff>

<commit_message>
test(validation): implement TC_LOGIN_10 for leading and trailing whitespace handling
</commit_message>
<xml_diff>
--- a/test-data/LoginTestCases.xlsx
+++ b/test-data/LoginTestCases.xlsx
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -882,6 +882,43 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Đăng nhập với Tên đăng nhập chứa khoảng trắng ở đầu và cuối</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   student_test   </t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Utc@2026Password</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống xử lý cắt bỏ khoảng trắng hoặc từ chối đăng nhập an toàn</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống xử lý chuỗi có khoảng trắng an toàn và không gây lỗi cú pháp</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test(boundary): implement TC_LOGIN_11 for maximum input length boundary verification
</commit_message>
<xml_diff>
--- a/test-data/LoginTestCases.xlsx
+++ b/test-data/LoginTestCases.xlsx
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -919,6 +919,43 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Kiểm tra độ dài vượt ngưỡng tại ô Tên đăng nhập (Boundary Value)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>user_boundary_test_xxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxx</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Password@123</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống giới hạn độ dài hoặc từ chối dữ liệu vượt ngưỡng, không gây lỗi máy chủ</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống xử lý chuỗi cực đại an toàn và duy trì trạng thái đăng nhập ổn định</t>
+        </is>
+      </c>
+      <c r="G12" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test(validation): implement TC_LOGIN_12 for special characters input validation
</commit_message>
<xml_diff>
--- a/test-data/LoginTestCases.xlsx
+++ b/test-data/LoginTestCases.xlsx
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -956,6 +956,43 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Đăng nhập với Tên đăng nhập chứa toàn ký tự đặc biệt</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>!@#$%^&amp;*()_+{}[]</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Password@123</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống từ chối xác thực tài khoản có định dạng không hợp lệ</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống từ chối tài khoản chứa ký tự đặc biệt và ở lại trang đăng nhập</t>
+        </is>
+      </c>
+      <c r="G13" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test(ui): implement TC_LOGIN_13 for password masking input type verification
</commit_message>
<xml_diff>
--- a/test-data/LoginTestCases.xlsx
+++ b/test-data/LoginTestCases.xlsx
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -993,6 +993,43 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Kiểm tra thuộc tính ẩn ký tự ô Mật khẩu (Password Masking UI)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>student_test</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>PasswordSecret123</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Trường mật khẩu có thuộc tính type='password' để che giấu ký tự bảo mật</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Trường mật khẩu đảm bảo thuộc tính type='password' và che giấu ký tự đúng chuẩn</t>
+        </is>
+      </c>
+      <c r="G14" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(readme): update test cases matrix and Excel results for all 13 scenarios
</commit_message>
<xml_diff>
--- a/test-data/LoginTestCases.xlsx
+++ b/test-data/LoginTestCases.xlsx
@@ -9,15 +9,18 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LoginTestCases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="0" uniqueCount="0"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="24">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -84,6 +87,84 @@
       <b val="1"/>
       <color indexed="17"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
     </font>
   </fonts>
   <fills count="3">
@@ -126,7 +207,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -151,6 +232,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -519,13 +613,13 @@
   <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col min="1" max="1" customWidth="true" width="16.0"/>
+    <col min="2" max="2" customWidth="true" width="46.0"/>
+    <col min="3" max="3" customWidth="true" width="24.0"/>
+    <col min="4" max="4" customWidth="true" width="24.0"/>
+    <col min="5" max="5" customWidth="true" width="52.0"/>
+    <col min="6" max="6" customWidth="true" width="38.0"/>
+    <col min="7" max="7" customWidth="true" width="14.0"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -592,11 +686,13 @@
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
+        <v>Chuyển hướng thành công tới hệ thống, URL: https://vanphongdientu.utc.edu.vn/Login (Thông báo UI: Tài khoản hoặc mật khẩu không đúng.)</v>
         <is>
           <t>Chuyển hướng thành công tới hệ thống, URL: https://vanphongdientu.utc.edu.vn/Login</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="14" t="inlineStr">
+        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -629,11 +725,13 @@
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
+        <v>Hệ thống từ chối truy cập và ở lại trang đăng nhập do sai mật khẩu (Thông báo UI: Tài khoản hoặc mật khẩu không đúng.)</v>
         <is>
           <t>Hệ thống từ chối truy cập và ở lại trang đăng nhập do sai mật khẩu</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" s="15" t="inlineStr">
+        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -666,11 +764,13 @@
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
+        <v>Hệ thống từ chối xác thực tài khoản không tồn tại (Thông báo UI: Tài khoản hoặc mật khẩu không đúng.)</v>
         <is>
           <t>Hệ thống từ chối xác thực tài khoản không tồn tại</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="16" t="inlineStr">
+        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -695,11 +795,13 @@
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
+        <v>Không cho phép gửi form rỗng, hiển thị cảnh báo validation (Thông báo UI: Bạn chưa nhập tên đăng nhập)</v>
         <is>
           <t>Không cho phép gửi form rỗng, hiển thị cảnh báo validation</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="G5" s="17" t="inlineStr">
+        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -728,11 +830,13 @@
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
+        <v>Chặn gửi form rỗng mật khẩu, hiển thị cảnh báo hợp lệ (Thông báo UI: Bạn chưa nhập mật khẩu)</v>
         <is>
           <t>Chặn gửi form rỗng mật khẩu, hiển thị cảnh báo hợp lệ</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="G6" s="18" t="inlineStr">
+        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -761,11 +865,13 @@
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
+        <v>Chặn gửi form rỗng tên đăng nhập, hiển thị cảnh báo hợp lệ (Thông báo UI: Bạn chưa nhập tên đăng nhập)</v>
         <is>
           <t>Chặn gửi form rỗng tên đăng nhập, hiển thị cảnh báo hợp lệ</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="G7" s="19" t="inlineStr">
+        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -798,11 +904,13 @@
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
+        <v>Tích chọn ghi nhớ thành công và gửi dữ liệu đăng nhập hợp lệ (Thông báo UI: Tài khoản hoặc mật khẩu không đúng.)</v>
         <is>
           <t>Tích chọn ghi nhớ thành công và gửi dữ liệu đăng nhập hợp lệ</t>
         </is>
       </c>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="G8" s="20" t="inlineStr">
+        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -835,11 +943,13 @@
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
+        <v>Hệ thống ngăn chặn chuỗi payload SQL Injection an toàn (Thông báo UI: Tài khoản hoặc mật khẩu không đúng.)</v>
         <is>
           <t>Hệ thống ngăn chặn chuỗi payload SQL Injection an toàn</t>
         </is>
       </c>
-      <c r="G9" s="11" t="inlineStr">
+      <c r="G9" s="21" t="inlineStr">
+        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -872,11 +982,13 @@
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
+        <v>Hệ thống xử lý an toàn chuỗi XSS payload và từ chối xác thực (Thông báo UI: Tài khoản hoặc mật khẩu không đúng.)</v>
         <is>
           <t>Hệ thống xử lý an toàn chuỗi XSS payload và từ chối xác thực</t>
         </is>
       </c>
-      <c r="G10" s="13" t="inlineStr">
+      <c r="G10" s="22" t="inlineStr">
+        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -909,11 +1021,13 @@
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
+        <v>Hệ thống xử lý chuỗi có khoảng trắng an toàn và không gây lỗi cú pháp (Thông báo UI: Tài khoản hoặc mật khẩu không đúng.)</v>
         <is>
           <t>Hệ thống xử lý chuỗi có khoảng trắng an toàn và không gây lỗi cú pháp</t>
         </is>
       </c>
-      <c r="G11" s="13" t="inlineStr">
+      <c r="G11" s="23" t="inlineStr">
+        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -946,11 +1060,13 @@
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
+        <v>Hệ thống xử lý chuỗi cực đại an toàn và duy trì trạng thái đăng nhập ổn định (Thông báo UI: Tài khoản hoặc mật khẩu không đúng.)</v>
         <is>
           <t>Hệ thống xử lý chuỗi cực đại an toàn và duy trì trạng thái đăng nhập ổn định</t>
         </is>
       </c>
-      <c r="G12" s="13" t="inlineStr">
+      <c r="G12" s="24" t="inlineStr">
+        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -983,11 +1099,13 @@
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
+        <v>Hệ thống từ chối tài khoản chứa ký tự đặc biệt và ở lại trang đăng nhập (Thông báo UI: Tài khoản hoặc mật khẩu không đúng.)</v>
         <is>
           <t>Hệ thống từ chối tài khoản chứa ký tự đặc biệt và ở lại trang đăng nhập</t>
         </is>
       </c>
-      <c r="G13" s="13" t="inlineStr">
+      <c r="G13" s="25" t="inlineStr">
+        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>
@@ -1020,11 +1138,13 @@
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
+        <v>Trường mật khẩu đảm bảo thuộc tính type='password' và che giấu ký tự đúng chuẩn (Thông báo UI: Tài khoản hoặc mật khẩu không đúng.)</v>
         <is>
           <t>Trường mật khẩu đảm bảo thuộc tính type='password' và che giấu ký tự đúng chuẩn</t>
         </is>
       </c>
-      <c r="G14" s="13" t="inlineStr">
+      <c r="G14" s="26" t="inlineStr">
+        <v>PASS</v>
         <is>
           <t>PASS</t>
         </is>

</xml_diff>